<commit_message>
feat: implement accomplishment tracking page and report generation API with Excel export functionality
</commit_message>
<xml_diff>
--- a/context/AccomplishmentReportTemplate.xlsx
+++ b/context/AccomplishmentReportTemplate.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Intern-Hours\context\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{784AC68C-D659-4CE5-8250-F0FCF6D99DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449320F7-ECE2-4218-AA3B-D629C53ADB10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F72CC7CB-6248-4D0C-9336-70A564646807}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Accomplishment Report" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -103,7 +103,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -188,29 +188,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -242,32 +224,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -291,15 +252,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:colOff>200026</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>2</xdr:rowOff>
+      <xdr:rowOff>95252</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>102818</xdr:rowOff>
+      <xdr:colOff>200026</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>7568</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -329,7 +290,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1" y="2"/>
+          <a:off x="200026" y="95252"/>
           <a:ext cx="5486400" cy="864816"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -352,15 +313,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>149481</xdr:rowOff>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>187581</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>47624</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>85724</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -390,7 +351,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="0" y="9102981"/>
+          <a:off x="161925" y="8950581"/>
           <a:ext cx="5476875" cy="469643"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -412,16 +373,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>266701</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>266701</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>102816</xdr:rowOff>
+      <xdr:rowOff>140916</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -451,7 +412,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5486401" y="0"/>
+          <a:off x="6362701" y="38100"/>
           <a:ext cx="5486400" cy="864816"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -473,16 +434,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>149479</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>168529</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>600075</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>47622</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>66672</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -512,7 +473,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5495925" y="9102979"/>
+          <a:off x="6286500" y="8931529"/>
           <a:ext cx="5467350" cy="469643"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -832,10 +793,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65ED9DBE-6DB5-4D44-B30C-36F97EF741C4}">
-  <dimension ref="B7:Q46"/>
+  <dimension ref="B7:S46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C7" s="1" t="s">
         <v>0</v>
       </c>
@@ -843,23 +804,24 @@
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
-      <c r="K7" s="1" t="s">
+      <c r="L7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L7" s="1"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="K8" s="11" t="s">
+      <c r="M7" s="1"/>
+    </row>
+    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="L8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="13"/>
-    </row>
-    <row r="9" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="11"/>
+      <c r="S8" s="11"/>
+    </row>
+    <row r="9" spans="2:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C9" s="2" t="s">
         <v>1</v>
       </c>
@@ -867,15 +829,17 @@
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="15"/>
-      <c r="M9" s="15"/>
-      <c r="N9" s="15"/>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="16"/>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K9" s="12"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="11"/>
+      <c r="S9" s="11"/>
+    </row>
+    <row r="10" spans="2:19" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="s">
         <v>2</v>
       </c>
@@ -883,24 +847,28 @@
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="15"/>
-      <c r="M10" s="15"/>
-      <c r="N10" s="15"/>
-      <c r="O10" s="15"/>
-      <c r="P10" s="15"/>
-      <c r="Q10" s="16"/>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="K11" s="14"/>
-      <c r="L11" s="15"/>
-      <c r="M11" s="15"/>
-      <c r="N11" s="15"/>
-      <c r="O11" s="15"/>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="16"/>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K10" s="12"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="11"/>
+      <c r="S10" s="11"/>
+    </row>
+    <row r="11" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="K11" s="12"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>12</v>
       </c>
@@ -912,15 +880,17 @@
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="15"/>
-      <c r="M12" s="15"/>
-      <c r="N12" s="15"/>
-      <c r="O12" s="15"/>
-      <c r="P12" s="15"/>
-      <c r="Q12" s="16"/>
-    </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K12" s="12"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="11"/>
+      <c r="R12" s="11"/>
+      <c r="S12" s="11"/>
+    </row>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>11</v>
       </c>
@@ -932,15 +902,17 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="15"/>
-      <c r="M13" s="15"/>
-      <c r="N13" s="15"/>
-      <c r="O13" s="15"/>
-      <c r="P13" s="15"/>
-      <c r="Q13" s="16"/>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K13" s="12"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="11"/>
+      <c r="Q13" s="11"/>
+      <c r="R13" s="11"/>
+      <c r="S13" s="11"/>
+    </row>
+    <row r="14" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>17</v>
       </c>
@@ -952,24 +924,28 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15"/>
-      <c r="N14" s="15"/>
-      <c r="O14" s="15"/>
-      <c r="P14" s="15"/>
-      <c r="Q14" s="16"/>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="K15" s="14"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="15"/>
-      <c r="O15" s="15"/>
-      <c r="P15" s="15"/>
-      <c r="Q15" s="16"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K14" s="12"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="11"/>
+      <c r="S14" s="11"/>
+    </row>
+    <row r="15" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="K15" s="12"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="11"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="11"/>
+      <c r="S15" s="11"/>
+    </row>
+    <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
         <v>3</v>
       </c>
@@ -979,15 +955,17 @@
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15"/>
-      <c r="N16" s="15"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-      <c r="Q16" s="16"/>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K16" s="12"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="11"/>
+      <c r="P16" s="11"/>
+      <c r="Q16" s="11"/>
+      <c r="R16" s="11"/>
+      <c r="S16" s="11"/>
+    </row>
+    <row r="17" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B17" s="10">
         <v>1</v>
       </c>
@@ -997,15 +975,17 @@
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="15"/>
-      <c r="M17" s="15"/>
-      <c r="N17" s="15"/>
-      <c r="O17" s="15"/>
-      <c r="P17" s="15"/>
-      <c r="Q17" s="16"/>
-    </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K17" s="12"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="11"/>
+      <c r="P17" s="11"/>
+      <c r="Q17" s="11"/>
+      <c r="R17" s="11"/>
+      <c r="S17" s="11"/>
+    </row>
+    <row r="18" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B18" s="10">
         <v>2</v>
       </c>
@@ -1015,15 +995,17 @@
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="16"/>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K18" s="12"/>
+      <c r="L18" s="11"/>
+      <c r="M18" s="11"/>
+      <c r="N18" s="11"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="11"/>
+      <c r="Q18" s="11"/>
+      <c r="R18" s="11"/>
+      <c r="S18" s="11"/>
+    </row>
+    <row r="19" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B19" s="10">
         <v>3</v>
       </c>
@@ -1033,15 +1015,17 @@
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="15"/>
-      <c r="M19" s="15"/>
-      <c r="N19" s="15"/>
-      <c r="O19" s="15"/>
-      <c r="P19" s="15"/>
-      <c r="Q19" s="16"/>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K19" s="12"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="11"/>
+      <c r="O19" s="11"/>
+      <c r="P19" s="11"/>
+      <c r="Q19" s="11"/>
+      <c r="R19" s="11"/>
+      <c r="S19" s="11"/>
+    </row>
+    <row r="20" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B20" s="10">
         <v>4</v>
       </c>
@@ -1051,15 +1035,17 @@
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="15"/>
-      <c r="M20" s="15"/>
-      <c r="N20" s="15"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="16"/>
-    </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K20" s="12"/>
+      <c r="L20" s="11"/>
+      <c r="M20" s="11"/>
+      <c r="N20" s="11"/>
+      <c r="O20" s="11"/>
+      <c r="P20" s="11"/>
+      <c r="Q20" s="11"/>
+      <c r="R20" s="11"/>
+      <c r="S20" s="11"/>
+    </row>
+    <row r="21" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B21" s="10">
         <v>5</v>
       </c>
@@ -1069,24 +1055,28 @@
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="15"/>
-      <c r="M21" s="15"/>
-      <c r="N21" s="15"/>
-      <c r="O21" s="15"/>
-      <c r="P21" s="15"/>
-      <c r="Q21" s="16"/>
-    </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="K22" s="14"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
-      <c r="N22" s="15"/>
-      <c r="O22" s="15"/>
-      <c r="P22" s="15"/>
-      <c r="Q22" s="16"/>
-    </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K21" s="12"/>
+      <c r="L21" s="11"/>
+      <c r="M21" s="11"/>
+      <c r="N21" s="11"/>
+      <c r="O21" s="11"/>
+      <c r="P21" s="11"/>
+      <c r="Q21" s="11"/>
+      <c r="R21" s="11"/>
+      <c r="S21" s="11"/>
+    </row>
+    <row r="22" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="K22" s="12"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="11"/>
+      <c r="N22" s="11"/>
+      <c r="O22" s="11"/>
+      <c r="P22" s="11"/>
+      <c r="Q22" s="11"/>
+      <c r="R22" s="11"/>
+      <c r="S22" s="11"/>
+    </row>
+    <row r="23" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B23" s="3" t="s">
         <v>4</v>
       </c>
@@ -1098,15 +1088,17 @@
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="15"/>
-      <c r="M23" s="15"/>
-      <c r="N23" s="15"/>
-      <c r="O23" s="15"/>
-      <c r="P23" s="15"/>
-      <c r="Q23" s="16"/>
-    </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K23" s="12"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="11"/>
+      <c r="P23" s="11"/>
+      <c r="Q23" s="11"/>
+      <c r="R23" s="11"/>
+      <c r="S23" s="11"/>
+    </row>
+    <row r="24" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B24" s="4"/>
       <c r="C24" s="5"/>
       <c r="D24" s="6"/>
@@ -1114,15 +1106,17 @@
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
       <c r="H24" s="6"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="15"/>
-      <c r="M24" s="15"/>
-      <c r="N24" s="15"/>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-      <c r="Q24" s="16"/>
-    </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K24" s="12"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="11"/>
+      <c r="O24" s="11"/>
+      <c r="P24" s="11"/>
+      <c r="Q24" s="11"/>
+      <c r="R24" s="11"/>
+      <c r="S24" s="11"/>
+    </row>
+    <row r="25" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B25" s="7"/>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
@@ -1130,15 +1124,17 @@
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
       <c r="H25" s="9"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
-      <c r="N25" s="15"/>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="16"/>
-    </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K25" s="12"/>
+      <c r="L25" s="11"/>
+      <c r="M25" s="11"/>
+      <c r="N25" s="11"/>
+      <c r="O25" s="11"/>
+      <c r="P25" s="11"/>
+      <c r="Q25" s="11"/>
+      <c r="R25" s="11"/>
+      <c r="S25" s="11"/>
+    </row>
+    <row r="26" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B26" s="4"/>
       <c r="C26" s="5"/>
       <c r="D26" s="6"/>
@@ -1146,15 +1142,17 @@
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
       <c r="H26" s="6"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
-      <c r="N26" s="15"/>
-      <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
-      <c r="Q26" s="16"/>
-    </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K26" s="12"/>
+      <c r="L26" s="11"/>
+      <c r="M26" s="11"/>
+      <c r="N26" s="11"/>
+      <c r="O26" s="11"/>
+      <c r="P26" s="11"/>
+      <c r="Q26" s="11"/>
+      <c r="R26" s="11"/>
+      <c r="S26" s="11"/>
+    </row>
+    <row r="27" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B27" s="7"/>
       <c r="C27" s="8"/>
       <c r="D27" s="9"/>
@@ -1162,15 +1160,17 @@
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
       <c r="H27" s="9"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="15"/>
-      <c r="M27" s="15"/>
-      <c r="N27" s="15"/>
-      <c r="O27" s="15"/>
-      <c r="P27" s="15"/>
-      <c r="Q27" s="16"/>
-    </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K27" s="12"/>
+      <c r="L27" s="11"/>
+      <c r="M27" s="11"/>
+      <c r="N27" s="11"/>
+      <c r="O27" s="11"/>
+      <c r="P27" s="11"/>
+      <c r="Q27" s="11"/>
+      <c r="R27" s="11"/>
+      <c r="S27" s="11"/>
+    </row>
+    <row r="28" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B28" s="4"/>
       <c r="C28" s="5"/>
       <c r="D28" s="6"/>
@@ -1178,15 +1178,17 @@
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
       <c r="H28" s="6"/>
-      <c r="K28" s="14"/>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
-      <c r="N28" s="15"/>
-      <c r="O28" s="15"/>
-      <c r="P28" s="15"/>
-      <c r="Q28" s="16"/>
-    </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K28" s="12"/>
+      <c r="L28" s="11"/>
+      <c r="M28" s="11"/>
+      <c r="N28" s="11"/>
+      <c r="O28" s="11"/>
+      <c r="P28" s="11"/>
+      <c r="Q28" s="11"/>
+      <c r="R28" s="11"/>
+      <c r="S28" s="11"/>
+    </row>
+    <row r="29" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B29" s="7"/>
       <c r="C29" s="8"/>
       <c r="D29" s="9"/>
@@ -1194,15 +1196,17 @@
       <c r="F29" s="8"/>
       <c r="G29" s="8"/>
       <c r="H29" s="9"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="15"/>
-      <c r="M29" s="15"/>
-      <c r="N29" s="15"/>
-      <c r="O29" s="15"/>
-      <c r="P29" s="15"/>
-      <c r="Q29" s="16"/>
-    </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K29" s="12"/>
+      <c r="L29" s="11"/>
+      <c r="M29" s="11"/>
+      <c r="N29" s="11"/>
+      <c r="O29" s="11"/>
+      <c r="P29" s="11"/>
+      <c r="Q29" s="11"/>
+      <c r="R29" s="11"/>
+      <c r="S29" s="11"/>
+    </row>
+    <row r="30" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B30" s="4"/>
       <c r="C30" s="5"/>
       <c r="D30" s="6"/>
@@ -1210,15 +1214,17 @@
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
       <c r="H30" s="6"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="15"/>
-      <c r="M30" s="15"/>
-      <c r="N30" s="15"/>
-      <c r="O30" s="15"/>
-      <c r="P30" s="15"/>
-      <c r="Q30" s="16"/>
-    </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K30" s="12"/>
+      <c r="L30" s="11"/>
+      <c r="M30" s="11"/>
+      <c r="N30" s="11"/>
+      <c r="O30" s="11"/>
+      <c r="P30" s="11"/>
+      <c r="Q30" s="11"/>
+      <c r="R30" s="11"/>
+      <c r="S30" s="11"/>
+    </row>
+    <row r="31" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B31" s="7"/>
       <c r="C31" s="8"/>
       <c r="D31" s="9"/>
@@ -1226,15 +1232,17 @@
       <c r="F31" s="8"/>
       <c r="G31" s="8"/>
       <c r="H31" s="9"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="N31" s="15"/>
-      <c r="O31" s="15"/>
-      <c r="P31" s="15"/>
-      <c r="Q31" s="16"/>
-    </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K31" s="12"/>
+      <c r="L31" s="11"/>
+      <c r="M31" s="11"/>
+      <c r="N31" s="11"/>
+      <c r="O31" s="11"/>
+      <c r="P31" s="11"/>
+      <c r="Q31" s="11"/>
+      <c r="R31" s="11"/>
+      <c r="S31" s="11"/>
+    </row>
+    <row r="32" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B32" s="4"/>
       <c r="C32" s="5"/>
       <c r="D32" s="6"/>
@@ -1242,15 +1250,17 @@
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
       <c r="H32" s="6"/>
-      <c r="K32" s="14"/>
-      <c r="L32" s="15"/>
-      <c r="M32" s="15"/>
-      <c r="N32" s="15"/>
-      <c r="O32" s="15"/>
-      <c r="P32" s="15"/>
-      <c r="Q32" s="16"/>
-    </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K32" s="12"/>
+      <c r="L32" s="11"/>
+      <c r="M32" s="11"/>
+      <c r="N32" s="11"/>
+      <c r="O32" s="11"/>
+      <c r="P32" s="11"/>
+      <c r="Q32" s="11"/>
+      <c r="R32" s="11"/>
+      <c r="S32" s="11"/>
+    </row>
+    <row r="33" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B33" s="7"/>
       <c r="C33" s="8"/>
       <c r="D33" s="9"/>
@@ -1258,15 +1268,17 @@
       <c r="F33" s="8"/>
       <c r="G33" s="8"/>
       <c r="H33" s="9"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="15"/>
-      <c r="M33" s="15"/>
-      <c r="N33" s="15"/>
-      <c r="O33" s="15"/>
-      <c r="P33" s="15"/>
-      <c r="Q33" s="16"/>
-    </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K33" s="12"/>
+      <c r="L33" s="11"/>
+      <c r="M33" s="11"/>
+      <c r="N33" s="11"/>
+      <c r="O33" s="11"/>
+      <c r="P33" s="11"/>
+      <c r="Q33" s="11"/>
+      <c r="R33" s="11"/>
+      <c r="S33" s="11"/>
+    </row>
+    <row r="34" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B34" s="4"/>
       <c r="C34" s="5"/>
       <c r="D34" s="6"/>
@@ -1274,15 +1286,17 @@
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
       <c r="H34" s="6"/>
-      <c r="K34" s="14"/>
-      <c r="L34" s="15"/>
-      <c r="M34" s="15"/>
-      <c r="N34" s="15"/>
-      <c r="O34" s="15"/>
-      <c r="P34" s="15"/>
-      <c r="Q34" s="16"/>
-    </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K34" s="12"/>
+      <c r="L34" s="11"/>
+      <c r="M34" s="11"/>
+      <c r="N34" s="11"/>
+      <c r="O34" s="11"/>
+      <c r="P34" s="11"/>
+      <c r="Q34" s="11"/>
+      <c r="R34" s="11"/>
+      <c r="S34" s="11"/>
+    </row>
+    <row r="35" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B35" s="7"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
@@ -1290,15 +1304,17 @@
       <c r="F35" s="8"/>
       <c r="G35" s="8"/>
       <c r="H35" s="9"/>
-      <c r="K35" s="14"/>
-      <c r="L35" s="15"/>
-      <c r="M35" s="15"/>
-      <c r="N35" s="15"/>
-      <c r="O35" s="15"/>
-      <c r="P35" s="15"/>
-      <c r="Q35" s="16"/>
-    </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K35" s="12"/>
+      <c r="L35" s="11"/>
+      <c r="M35" s="11"/>
+      <c r="N35" s="11"/>
+      <c r="O35" s="11"/>
+      <c r="P35" s="11"/>
+      <c r="Q35" s="11"/>
+      <c r="R35" s="11"/>
+      <c r="S35" s="11"/>
+    </row>
+    <row r="36" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B36" s="4"/>
       <c r="C36" s="5"/>
       <c r="D36" s="6"/>
@@ -1306,15 +1322,17 @@
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
       <c r="H36" s="6"/>
-      <c r="K36" s="14"/>
-      <c r="L36" s="15"/>
-      <c r="M36" s="15"/>
-      <c r="N36" s="15"/>
-      <c r="O36" s="15"/>
-      <c r="P36" s="15"/>
-      <c r="Q36" s="16"/>
-    </row>
-    <row r="37" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K36" s="12"/>
+      <c r="L36" s="11"/>
+      <c r="M36" s="11"/>
+      <c r="N36" s="11"/>
+      <c r="O36" s="11"/>
+      <c r="P36" s="11"/>
+      <c r="Q36" s="11"/>
+      <c r="R36" s="11"/>
+      <c r="S36" s="11"/>
+    </row>
+    <row r="37" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B37" s="7"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
@@ -1322,15 +1340,17 @@
       <c r="F37" s="8"/>
       <c r="G37" s="8"/>
       <c r="H37" s="9"/>
-      <c r="K37" s="14"/>
-      <c r="L37" s="15"/>
-      <c r="M37" s="15"/>
-      <c r="N37" s="15"/>
-      <c r="O37" s="15"/>
-      <c r="P37" s="15"/>
-      <c r="Q37" s="16"/>
-    </row>
-    <row r="38" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K37" s="12"/>
+      <c r="L37" s="11"/>
+      <c r="M37" s="11"/>
+      <c r="N37" s="11"/>
+      <c r="O37" s="11"/>
+      <c r="P37" s="11"/>
+      <c r="Q37" s="11"/>
+      <c r="R37" s="11"/>
+      <c r="S37" s="11"/>
+    </row>
+    <row r="38" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B38" s="4"/>
       <c r="C38" s="5"/>
       <c r="D38" s="6"/>
@@ -1338,15 +1358,17 @@
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
       <c r="H38" s="6"/>
-      <c r="K38" s="17"/>
-      <c r="L38" s="18"/>
-      <c r="M38" s="18"/>
-      <c r="N38" s="18"/>
-      <c r="O38" s="18"/>
-      <c r="P38" s="18"/>
-      <c r="Q38" s="19"/>
-    </row>
-    <row r="39" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="K38" s="12"/>
+      <c r="L38" s="11"/>
+      <c r="M38" s="11"/>
+      <c r="N38" s="11"/>
+      <c r="O38" s="11"/>
+      <c r="P38" s="11"/>
+      <c r="Q38" s="11"/>
+      <c r="R38" s="11"/>
+      <c r="S38" s="11"/>
+    </row>
+    <row r="39" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B39" s="7"/>
       <c r="C39" s="8"/>
       <c r="D39" s="9"/>
@@ -1355,7 +1377,7 @@
       <c r="G39" s="8"/>
       <c r="H39" s="9"/>
     </row>
-    <row r="40" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -1363,11 +1385,11 @@
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
-      <c r="K40" t="s">
+      <c r="L40" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -1375,14 +1397,14 @@
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
-      <c r="K41" s="8"/>
       <c r="L41" s="8"/>
       <c r="M41" s="8"/>
-      <c r="O41" s="8"/>
+      <c r="N41" s="8"/>
       <c r="P41" s="8"/>
       <c r="Q41" s="8"/>
-    </row>
-    <row r="42" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="R41" s="8"/>
+    </row>
+    <row r="42" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
@@ -1390,18 +1412,18 @@
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
-      <c r="K42" s="1" t="s">
+      <c r="L42" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L42" s="1"/>
-      <c r="M42" s="1"/>
-      <c r="O42" s="1" t="s">
+      <c r="M42" s="5"/>
+      <c r="N42" s="5"/>
+      <c r="P42" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="P42" s="1"/>
-      <c r="Q42" s="1"/>
-    </row>
-    <row r="43" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q42" s="5"/>
+      <c r="R42" s="5"/>
+    </row>
+    <row r="43" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
@@ -1410,7 +1432,7 @@
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
     </row>
-    <row r="44" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
@@ -1419,7 +1441,7 @@
       <c r="G44" s="3"/>
       <c r="H44" s="3"/>
     </row>
-    <row r="45" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
@@ -1427,29 +1449,29 @@
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
-      <c r="K45" s="8"/>
       <c r="L45" s="8"/>
       <c r="M45" s="8"/>
-    </row>
-    <row r="46" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="K46" s="1" t="s">
+      <c r="N45" s="8"/>
+    </row>
+    <row r="46" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="L46" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="L46" s="1"/>
-      <c r="M46" s="1"/>
+      <c r="M46" s="5"/>
+      <c r="N46" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="K46:M46"/>
-    <mergeCell ref="K8:Q38"/>
+    <mergeCell ref="L7:M7"/>
+    <mergeCell ref="L8:S38"/>
+    <mergeCell ref="P42:R42"/>
+    <mergeCell ref="L42:N42"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="L45:N45"/>
+    <mergeCell ref="L41:N41"/>
+    <mergeCell ref="P41:R41"/>
     <mergeCell ref="E44:H45"/>
     <mergeCell ref="B44:D45"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="K41:M41"/>
-    <mergeCell ref="O41:Q41"/>
-    <mergeCell ref="K42:M42"/>
-    <mergeCell ref="O42:Q42"/>
-    <mergeCell ref="K45:M45"/>
     <mergeCell ref="E30:H31"/>
     <mergeCell ref="E28:H29"/>
     <mergeCell ref="E26:H27"/>
@@ -1488,7 +1510,7 @@
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="B12:C12"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>